<commit_message>
removing colours from cells and adding some missing dates
</commit_message>
<xml_diff>
--- a/auxiliary-data/Soil properties.xlsx
+++ b/auxiliary-data/Soil properties.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="8" documentId="8_{C72C030A-5F10-4045-AB61-9DBFC8374B6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A62F551C-F077-4B97-A435-45E7C4AA7956}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="8_{C72C030A-5F10-4045-AB61-9DBFC8374B6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4E1A2CC2-8DD8-4174-B01D-3FBD0096C7EF}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1211,6 +1211,9 @@
       <c r="A19">
         <v>8</v>
       </c>
+      <c r="B19">
+        <v>220921</v>
+      </c>
       <c r="C19">
         <v>2</v>
       </c>
@@ -1248,6 +1251,9 @@
     <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>8</v>
+      </c>
+      <c r="B20">
+        <v>220921</v>
       </c>
       <c r="C20">
         <v>3</v>
@@ -1325,6 +1331,9 @@
       <c r="A22">
         <v>7</v>
       </c>
+      <c r="B22">
+        <v>220928</v>
+      </c>
       <c r="C22">
         <v>2</v>
       </c>
@@ -1363,6 +1372,9 @@
       <c r="A23">
         <v>7</v>
       </c>
+      <c r="B23">
+        <v>220928</v>
+      </c>
       <c r="C23">
         <v>3</v>
       </c>
@@ -1439,6 +1451,9 @@
       <c r="A25">
         <v>6</v>
       </c>
+      <c r="B25">
+        <v>221019</v>
+      </c>
       <c r="C25">
         <v>2</v>
       </c>
@@ -1477,6 +1492,9 @@
       <c r="A26">
         <v>6</v>
       </c>
+      <c r="B26">
+        <v>221019</v>
+      </c>
       <c r="C26">
         <v>3</v>
       </c>
@@ -1553,6 +1571,9 @@
       <c r="A28">
         <v>9</v>
       </c>
+      <c r="B28">
+        <v>221025</v>
+      </c>
       <c r="C28">
         <v>2</v>
       </c>
@@ -1590,6 +1611,9 @@
     <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>9</v>
+      </c>
+      <c r="B29">
+        <v>221025</v>
       </c>
       <c r="C29">
         <v>3</v>
@@ -1646,4 +1670,10 @@
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7408D0D6-C97A-426B-8466-DDDAA7A3F420}">
   <ds:schemaRefs/>
 </ds:datastoreItem>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{61fd1d36-fecb-47ca-b7d7-d0df0370a198}" enabled="0" method="" siteId="{61fd1d36-fecb-47ca-b7d7-d0df0370a198}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>